<commit_message>
feat: add new report in excell file
</commit_message>
<xml_diff>
--- a/Api/wwwroot/GetReportSymptoms.xlsx
+++ b/Api/wwwroot/GetReportSymptoms.xlsx
@@ -11,13 +11,15 @@
     <sheet name="Patient_somi" sheetId="4" r:id="rId5"/>
     <sheet name="Patient_Zahra" sheetId="5" r:id="rId6"/>
     <sheet name="Symptoms Overview" sheetId="6" r:id="rId7"/>
+    <sheet name="Symptom Matrix" sheetId="7" r:id="rId8"/>
+    <sheet name="Symptom Week Matrix" sheetId="8" r:id="rId9"/>
   </sheets>
   <calcPr fullCalcOnLoad="1" fullPrecision="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="86">
   <si>
     <t>Patient Summary Report</t>
   </si>
@@ -227,6 +229,54 @@
   </si>
   <si>
     <t>Min Degree</t>
+  </si>
+  <si>
+    <t>Symptom \ Patient</t>
+  </si>
+  <si>
+    <t>week1, week2, week3, week4, week5, week6, week7, week8, week9</t>
+  </si>
+  <si>
+    <t>week1</t>
+  </si>
+  <si>
+    <t>week1, week2</t>
+  </si>
+  <si>
+    <t>week1, week2, week3, week4, week5, week6, week7, week8</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>week1, week2, week3, week4</t>
+  </si>
+  <si>
+    <t>week1, week2, week3</t>
+  </si>
+  <si>
+    <t>Symptom Name</t>
+  </si>
+  <si>
+    <t>Week 1</t>
+  </si>
+  <si>
+    <t>Week 2</t>
+  </si>
+  <si>
+    <t>Week 3</t>
+  </si>
+  <si>
+    <t>Week 4</t>
+  </si>
+  <si>
+    <t>Week 5</t>
+  </si>
+  <si>
+    <t>Week 6</t>
+  </si>
+  <si>
+    <t>Week 7</t>
   </si>
 </sst>
 </file>
@@ -275,7 +325,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="2" applyFont="1" applyAlignment="1">
@@ -283,6 +333,9 @@
     </xf>
     <xf numFmtId="0" fontId="3" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -490,7 +543,7 @@
         <v>24</v>
       </c>
       <c r="E6" s="0">
-        <v>301</v>
+        <v>302</v>
       </c>
     </row>
     <row r="7">
@@ -507,7 +560,7 @@
         <v>26</v>
       </c>
       <c r="E7" s="0">
-        <v>294</v>
+        <v>295</v>
       </c>
     </row>
     <row r="8">
@@ -524,7 +577,7 @@
         <v>28</v>
       </c>
       <c r="E8" s="0">
-        <v>287</v>
+        <v>288</v>
       </c>
     </row>
     <row r="9">
@@ -541,7 +594,7 @@
         <v>29</v>
       </c>
       <c r="E9" s="0">
-        <v>280</v>
+        <v>281</v>
       </c>
     </row>
     <row r="10">
@@ -558,7 +611,7 @@
         <v>31</v>
       </c>
       <c r="E10" s="0">
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
     <row r="11">
@@ -575,7 +628,7 @@
         <v>31</v>
       </c>
       <c r="E11" s="0">
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
     <row r="12">
@@ -592,7 +645,7 @@
         <v>33</v>
       </c>
       <c r="E12" s="0">
-        <v>266</v>
+        <v>267</v>
       </c>
     </row>
     <row r="13">
@@ -609,7 +662,7 @@
         <v>34</v>
       </c>
       <c r="E13" s="0">
-        <v>259</v>
+        <v>260</v>
       </c>
     </row>
     <row r="15">
@@ -665,7 +718,7 @@
         <v>36</v>
       </c>
       <c r="E18" s="0">
-        <v>302</v>
+        <v>303</v>
       </c>
     </row>
     <row r="19">
@@ -682,7 +735,7 @@
         <v>36</v>
       </c>
       <c r="E19" s="0">
-        <v>302</v>
+        <v>303</v>
       </c>
     </row>
     <row r="20">
@@ -699,7 +752,7 @@
         <v>36</v>
       </c>
       <c r="E20" s="0">
-        <v>302</v>
+        <v>303</v>
       </c>
     </row>
     <row r="21">
@@ -716,7 +769,7 @@
         <v>37</v>
       </c>
       <c r="E21" s="0">
-        <v>295</v>
+        <v>296</v>
       </c>
     </row>
     <row r="22">
@@ -733,7 +786,7 @@
         <v>38</v>
       </c>
       <c r="E22" s="0">
-        <v>288</v>
+        <v>289</v>
       </c>
     </row>
     <row r="23">
@@ -750,7 +803,7 @@
         <v>40</v>
       </c>
       <c r="E23" s="0">
-        <v>281</v>
+        <v>282</v>
       </c>
     </row>
     <row r="24">
@@ -767,7 +820,7 @@
         <v>41</v>
       </c>
       <c r="E24" s="0">
-        <v>274</v>
+        <v>275</v>
       </c>
     </row>
     <row r="26">
@@ -806,7 +859,7 @@
         <v>34</v>
       </c>
       <c r="E28" s="0">
-        <v>259</v>
+        <v>260</v>
       </c>
     </row>
     <row r="30">
@@ -862,7 +915,7 @@
         <v>36</v>
       </c>
       <c r="E33" s="0">
-        <v>302</v>
+        <v>303</v>
       </c>
     </row>
     <row r="35">
@@ -901,7 +954,7 @@
         <v>36</v>
       </c>
       <c r="E37" s="0">
-        <v>302</v>
+        <v>303</v>
       </c>
     </row>
     <row r="39">
@@ -940,7 +993,7 @@
         <v>26</v>
       </c>
       <c r="E41" s="0">
-        <v>294</v>
+        <v>295</v>
       </c>
     </row>
   </sheetData>
@@ -1077,7 +1130,7 @@
         <v>51</v>
       </c>
       <c r="E5" s="0">
-        <v>66</v>
+        <v>67</v>
       </c>
     </row>
     <row r="7">
@@ -1116,7 +1169,7 @@
         <v>51</v>
       </c>
       <c r="E9" s="0">
-        <v>66</v>
+        <v>67</v>
       </c>
     </row>
     <row r="11">
@@ -1155,7 +1208,7 @@
         <v>51</v>
       </c>
       <c r="E13" s="0">
-        <v>66</v>
+        <v>67</v>
       </c>
     </row>
     <row r="15">
@@ -1194,7 +1247,7 @@
         <v>51</v>
       </c>
       <c r="E17" s="0">
-        <v>66</v>
+        <v>67</v>
       </c>
     </row>
     <row r="19">
@@ -1233,7 +1286,7 @@
         <v>51</v>
       </c>
       <c r="E21" s="0">
-        <v>66</v>
+        <v>67</v>
       </c>
     </row>
   </sheetData>
@@ -1303,7 +1356,7 @@
         <v>54</v>
       </c>
       <c r="E5" s="0">
-        <v>100</v>
+        <v>101</v>
       </c>
     </row>
     <row r="6">
@@ -1320,7 +1373,7 @@
         <v>56</v>
       </c>
       <c r="E6" s="0">
-        <v>94</v>
+        <v>95</v>
       </c>
     </row>
     <row r="8">
@@ -1359,7 +1412,7 @@
         <v>54</v>
       </c>
       <c r="E10" s="0">
-        <v>100</v>
+        <v>101</v>
       </c>
     </row>
     <row r="11">
@@ -1376,7 +1429,7 @@
         <v>56</v>
       </c>
       <c r="E11" s="0">
-        <v>94</v>
+        <v>95</v>
       </c>
     </row>
     <row r="12">
@@ -1393,7 +1446,7 @@
         <v>58</v>
       </c>
       <c r="E12" s="0">
-        <v>87</v>
+        <v>88</v>
       </c>
     </row>
     <row r="13">
@@ -1410,7 +1463,7 @@
         <v>59</v>
       </c>
       <c r="E13" s="0">
-        <v>80</v>
+        <v>81</v>
       </c>
     </row>
     <row r="15">
@@ -1449,7 +1502,7 @@
         <v>54</v>
       </c>
       <c r="E17" s="0">
-        <v>100</v>
+        <v>101</v>
       </c>
     </row>
     <row r="18">
@@ -1466,7 +1519,7 @@
         <v>56</v>
       </c>
       <c r="E18" s="0">
-        <v>94</v>
+        <v>95</v>
       </c>
     </row>
     <row r="20">
@@ -1505,7 +1558,7 @@
         <v>54</v>
       </c>
       <c r="E22" s="0">
-        <v>100</v>
+        <v>101</v>
       </c>
     </row>
     <row r="23">
@@ -1522,7 +1575,7 @@
         <v>56</v>
       </c>
       <c r="E23" s="0">
-        <v>94</v>
+        <v>95</v>
       </c>
     </row>
     <row r="24">
@@ -1539,7 +1592,7 @@
         <v>58</v>
       </c>
       <c r="E24" s="0">
-        <v>87</v>
+        <v>88</v>
       </c>
     </row>
     <row r="26">
@@ -1578,7 +1631,7 @@
         <v>54</v>
       </c>
       <c r="E28" s="0">
-        <v>100</v>
+        <v>101</v>
       </c>
     </row>
     <row r="29">
@@ -1595,7 +1648,7 @@
         <v>56</v>
       </c>
       <c r="E29" s="0">
-        <v>94</v>
+        <v>95</v>
       </c>
     </row>
     <row r="31">
@@ -1634,7 +1687,7 @@
         <v>54</v>
       </c>
       <c r="E33" s="0">
-        <v>100</v>
+        <v>101</v>
       </c>
     </row>
     <row r="34">
@@ -1651,7 +1704,7 @@
         <v>56</v>
       </c>
       <c r="E34" s="0">
-        <v>94</v>
+        <v>95</v>
       </c>
     </row>
     <row r="36">
@@ -1690,7 +1743,7 @@
         <v>54</v>
       </c>
       <c r="E38" s="0">
-        <v>100</v>
+        <v>101</v>
       </c>
     </row>
     <row r="39">
@@ -1707,7 +1760,7 @@
         <v>56</v>
       </c>
       <c r="E39" s="0">
-        <v>94</v>
+        <v>95</v>
       </c>
     </row>
     <row r="41">
@@ -1746,7 +1799,7 @@
         <v>54</v>
       </c>
       <c r="E43" s="0">
-        <v>100</v>
+        <v>101</v>
       </c>
     </row>
     <row r="44">
@@ -1763,7 +1816,7 @@
         <v>56</v>
       </c>
       <c r="E44" s="0">
-        <v>94</v>
+        <v>95</v>
       </c>
     </row>
   </sheetData>
@@ -1987,4 +2040,660 @@
   </mergeCells>
   <headerFooter/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr codeName=""/>
+  <dimension ref="A1:E9"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="60.72814178466797" customWidth="1"/>
+    <col min="2" max="2" width="60.801448822021484" customWidth="1"/>
+    <col min="3" max="3" width="9.140625" customWidth="1"/>
+    <col min="4" max="4" width="9.140625" customWidth="1"/>
+    <col min="5" max="5" width="26.840801239013672" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="0" t="s">
+        <v>70</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B2" s="0" t="s">
+        <v>71</v>
+      </c>
+      <c r="C2" s="0" t="s">
+        <v>72</v>
+      </c>
+      <c r="D2" s="0" t="s">
+        <v>72</v>
+      </c>
+      <c r="E2" s="0" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B3" s="0" t="s">
+        <v>74</v>
+      </c>
+      <c r="C3" s="0" t="s">
+        <v>75</v>
+      </c>
+      <c r="D3" s="0" t="s">
+        <v>75</v>
+      </c>
+      <c r="E3" s="0" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B4" s="0" t="s">
+        <v>72</v>
+      </c>
+      <c r="C4" s="0" t="s">
+        <v>75</v>
+      </c>
+      <c r="D4" s="0" t="s">
+        <v>72</v>
+      </c>
+      <c r="E4" s="0" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="B5" s="0" t="s">
+        <v>73</v>
+      </c>
+      <c r="C5" s="0" t="s">
+        <v>75</v>
+      </c>
+      <c r="D5" s="0" t="s">
+        <v>72</v>
+      </c>
+      <c r="E5" s="0" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="B6" s="0" t="s">
+        <v>72</v>
+      </c>
+      <c r="C6" s="0" t="s">
+        <v>75</v>
+      </c>
+      <c r="D6" s="0" t="s">
+        <v>72</v>
+      </c>
+      <c r="E6" s="0" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="B7" s="0" t="s">
+        <v>72</v>
+      </c>
+      <c r="C7" s="0" t="s">
+        <v>75</v>
+      </c>
+      <c r="D7" s="0" t="s">
+        <v>72</v>
+      </c>
+      <c r="E7" s="0" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="B8" s="0" t="s">
+        <v>75</v>
+      </c>
+      <c r="C8" s="0" t="s">
+        <v>75</v>
+      </c>
+      <c r="D8" s="0" t="s">
+        <v>75</v>
+      </c>
+      <c r="E8" s="0" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="B9" s="0" t="s">
+        <v>75</v>
+      </c>
+      <c r="C9" s="0" t="s">
+        <v>75</v>
+      </c>
+      <c r="D9" s="0" t="s">
+        <v>75</v>
+      </c>
+      <c r="E9" s="0" t="s">
+        <v>73</v>
+      </c>
+    </row>
+  </sheetData>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr codeName=""/>
+  <dimension ref="A1:F57"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="14.821828842163086" customWidth="1"/>
+    <col min="2" max="2" width="9.140625" customWidth="1"/>
+    <col min="3" max="3" width="9.140625" customWidth="1"/>
+    <col min="4" max="4" width="9.140625" customWidth="1"/>
+    <col min="5" max="5" width="9.140625" customWidth="1"/>
+    <col min="6" max="6" width="9.140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="0" t="s">
+        <v>78</v>
+      </c>
+      <c r="B1" s="0" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B2" s="0" t="s">
+        <v>79</v>
+      </c>
+      <c r="C2" s="0">
+        <v>7</v>
+      </c>
+      <c r="D2" s="0">
+        <v>8</v>
+      </c>
+      <c r="E2" s="0">
+        <v>0</v>
+      </c>
+      <c r="F2" s="0">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" s="0" t="s">
+        <v>80</v>
+      </c>
+      <c r="C3" s="0">
+        <v>10</v>
+      </c>
+      <c r="F3" s="0">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" s="0" t="s">
+        <v>81</v>
+      </c>
+      <c r="C4" s="0">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" s="0" t="s">
+        <v>82</v>
+      </c>
+      <c r="C5" s="0">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" s="0" t="s">
+        <v>83</v>
+      </c>
+      <c r="C6" s="0">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" s="0" t="s">
+        <v>84</v>
+      </c>
+      <c r="C7" s="0">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="0" t="s">
+        <v>85</v>
+      </c>
+      <c r="C8" s="0">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="B9" s="0" t="s">
+        <v>79</v>
+      </c>
+      <c r="C9" s="0">
+        <v>7</v>
+      </c>
+      <c r="F9" s="0">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="0" t="s">
+        <v>80</v>
+      </c>
+      <c r="C10" s="0">
+        <v>6</v>
+      </c>
+      <c r="F10" s="0">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" s="0" t="s">
+        <v>81</v>
+      </c>
+      <c r="C11" s="0">
+        <v>6</v>
+      </c>
+      <c r="F11" s="0">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="0" t="s">
+        <v>82</v>
+      </c>
+      <c r="C12" s="0">
+        <v>6</v>
+      </c>
+      <c r="F12" s="0">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" s="0" t="s">
+        <v>83</v>
+      </c>
+      <c r="C13" s="0">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="0" t="s">
+        <v>84</v>
+      </c>
+      <c r="C14" s="0">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="0" t="s">
+        <v>85</v>
+      </c>
+      <c r="C15" s="0">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="B16" s="0" t="s">
+        <v>79</v>
+      </c>
+      <c r="C16" s="0">
+        <v>6</v>
+      </c>
+      <c r="E16" s="0">
+        <v>7</v>
+      </c>
+      <c r="F16" s="0">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="0" t="s">
+        <v>80</v>
+      </c>
+      <c r="F17" s="0">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="0" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="0" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="0" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" s="0" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" s="0" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="B23" s="0" t="s">
+        <v>79</v>
+      </c>
+      <c r="C23" s="0">
+        <v>7</v>
+      </c>
+      <c r="E23" s="0">
+        <v>7</v>
+      </c>
+      <c r="F23" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="0" t="s">
+        <v>80</v>
+      </c>
+      <c r="C24" s="0">
+        <v>7</v>
+      </c>
+      <c r="F24" s="0">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" s="0" t="s">
+        <v>81</v>
+      </c>
+      <c r="F25" s="0">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" s="0" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" s="0" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" s="0" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" s="0" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="B30" s="0" t="s">
+        <v>79</v>
+      </c>
+      <c r="C30" s="0">
+        <v>6</v>
+      </c>
+      <c r="E30" s="0">
+        <v>7</v>
+      </c>
+      <c r="F30" s="0">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" s="0" t="s">
+        <v>80</v>
+      </c>
+      <c r="F31" s="0">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="B32" s="0" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="B33" s="0" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="B34" s="0" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="B35" s="0" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="B36" s="0" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="B37" s="0" t="s">
+        <v>79</v>
+      </c>
+      <c r="C37" s="0">
+        <v>7</v>
+      </c>
+      <c r="E37" s="0">
+        <v>0</v>
+      </c>
+      <c r="F37" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="B38" s="0" t="s">
+        <v>80</v>
+      </c>
+      <c r="F38" s="0">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="B39" s="0" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="B40" s="0" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="B41" s="0" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="B42" s="0" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="B43" s="0" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="B44" s="0" t="s">
+        <v>79</v>
+      </c>
+      <c r="F44" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="B45" s="0" t="s">
+        <v>80</v>
+      </c>
+      <c r="F45" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="B46" s="0" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="B47" s="0" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="B48" s="0" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="B49" s="0" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="B50" s="0" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="B51" s="0" t="s">
+        <v>79</v>
+      </c>
+      <c r="F51" s="0">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="B52" s="0" t="s">
+        <v>80</v>
+      </c>
+      <c r="F52" s="0">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="B53" s="0" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="B54" s="0" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="B55" s="0" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="B56" s="0" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="B57" s="0" t="s">
+        <v>85</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells>
+    <mergeCell ref="A2:A8"/>
+    <mergeCell ref="A9:A15"/>
+    <mergeCell ref="A16:A22"/>
+    <mergeCell ref="A23:A29"/>
+    <mergeCell ref="A30:A36"/>
+    <mergeCell ref="A37:A43"/>
+    <mergeCell ref="A44:A50"/>
+    <mergeCell ref="A51:A57"/>
+  </mergeCells>
+  <headerFooter/>
+</worksheet>
 </file>
</xml_diff>